<commit_message>
feat(comenzi-externe): simplified anexa template, flexible import parser, contract edit
- New 4-column anexa template: Nr. Comanda, Model, Color, VIN (VIN optional)
- Import parser rewritten with auto-detect headers, handles simple and full formats
- Contract edit endpoint (PATCH) for contract_ref, date, responsible, notes
- Template download link always visible on New Anexa dialog

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jarvis/accounting/facturare/assets/Anexa_Template.xlsx
+++ b/jarvis/accounting/facturare/assets/Anexa_Template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +28,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -73,18 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,217 +439,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ANEXA - Template Facturare</t>
+          <t>Nr. Comanda</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>VIN</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Comanda</t>
+          <t>151100</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Audi Q5 40 TFSI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Culoare</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Pret Lista</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Pret Vanzare</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Discount</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Avans (EUR)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Rest</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>VIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>509805</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Golf 8 1.5 TSI Life</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Pure White</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>25390</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>23500</v>
-      </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="4" t="n">
-        <v>2053</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>21447</v>
-      </c>
-      <c r="I3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>509806</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Golf 8 2.0 TDI Style</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Dolphin Grey</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>28750</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>26800</v>
-      </c>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="4" t="n">
-        <v>2150</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>24650</v>
-      </c>
-      <c r="I4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>150404</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Audi Q5 Sportback 40 TDI quattro</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Gri Daytona perlat</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>WAUZZZGU5S2121296</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>150411</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Audi Q5 Sportback 40 TDI quattro</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Gri Daytona perlat</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>WAUZZZGU6S2123719</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>150414</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Audi Q5 Sportback 40 TDI quattro</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Alb Gletscher Metalizat</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>WAUZZZGU4S2119524</t>
-        </is>
-      </c>
+          <t>Negru Mythos metalizat</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(comenzi-externe): add Pret Vanzare to import template, fix column detection
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jarvis/accounting/facturare/assets/Anexa_Template.xlsx
+++ b/jarvis/accounting/facturare/assets/Anexa_Template.xlsx
@@ -439,13 +439,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,12 +462,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>Culoare</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>VIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Pret Vanzare</t>
         </is>
       </c>
     </row>
@@ -487,6 +493,9 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n">
+        <v>38900</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>